<commit_message>
Use accented Vietnamese in comments and scenarios
</commit_message>
<xml_diff>
--- a/Output_2027/bao_cao_du_bao_2027.xlsx
+++ b/Output_2027/bao_cao_du_bao_2027.xlsx
@@ -536,17 +536,17 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Trung binh gan han + trung binh lich su + xu the + tham chieu 2025</t>
+          <t>Trung bình gần hạn + trung bình lịch sử + xu thế + tham chiếu 2025</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Chua co tan suat 2027, dung mo hinh bo sung</t>
+          <t>Chưa có tần suất 2027, dùng mô hình bổ sung</t>
         </is>
       </c>
     </row>
@@ -581,17 +581,17 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Trung binh gan han + trung binh lich su + xu the + tham chieu 2025</t>
+          <t>Trung bình gần hạn + trung bình lịch sử + xu thế + tham chiếu 2025</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Chua co tan suat 2027, dung mo hinh bo sung</t>
+          <t>Chưa có tần suất 2027, dùng mô hình bổ sung</t>
         </is>
       </c>
     </row>
@@ -626,17 +626,17 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Trung binh gan han + trung binh lich su + xu the + tham chieu 2025</t>
+          <t>Trung bình gần hạn + trung bình lịch sử + xu thế + tham chiếu 2025</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Chua co tan suat 2027, dung mo hinh bo sung</t>
+          <t>Chưa có tần suất 2027, dùng mô hình bổ sung</t>
         </is>
       </c>
     </row>
@@ -671,17 +671,17 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Nhieu nuoc</t>
+          <t>Nhiều nước</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Trung binh gan han + trung binh lich su + xu the + tham chieu 2025</t>
+          <t>Trung bình gần hạn + trung bình lịch sử + xu thế + tham chiếu 2025</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Chua co tan suat 2027, dung mo hinh bo sung</t>
+          <t>Chưa có tần suất 2027, dùng mô hình bổ sung</t>
         </is>
       </c>
     </row>
@@ -716,17 +716,17 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Nhieu nuoc</t>
+          <t>Nhiều nước</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Trung binh gan han + trung binh lich su + xu the + tham chieu 2025</t>
+          <t>Trung bình gần hạn + trung bình lịch sử + xu thế + tham chiếu 2025</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Chua co tan suat 2027, dung mo hinh bo sung</t>
+          <t>Chưa có tần suất 2027, dùng mô hình bổ sung</t>
         </is>
       </c>
     </row>
@@ -761,17 +761,17 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Nhieu nuoc</t>
+          <t>Nhiều nước</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Trung binh gan han + trung binh lich su + xu the + tham chieu 2025</t>
+          <t>Trung bình gần hạn + trung bình lịch sử + xu thế + tham chiếu 2025</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Chua co tan suat 2027, dung mo hinh bo sung</t>
+          <t>Chưa có tần suất 2027, dùng mô hình bổ sung</t>
         </is>
       </c>
     </row>
@@ -806,17 +806,17 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Nhieu nuoc</t>
+          <t>Nhiều nước</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Trung binh gan han + trung binh lich su + xu the + tham chieu 2025</t>
+          <t>Trung bình gần hạn + trung bình lịch sử + xu thế + tham chiếu 2025</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Chua co tan suat 2027, dung mo hinh bo sung</t>
+          <t>Chưa có tần suất 2027, dùng mô hình bổ sung</t>
         </is>
       </c>
     </row>
@@ -851,17 +851,17 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Trung binh gan han + trung binh lich su + xu the + tham chieu 2025</t>
+          <t>Trung bình gần hạn + trung bình lịch sử + xu thế + tham chiếu 2025</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Chua co tan suat 2027, dung mo hinh bo sung</t>
+          <t>Chưa có tần suất 2027, dùng mô hình bổ sung</t>
         </is>
       </c>
     </row>
@@ -896,17 +896,17 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Nhieu nuoc</t>
+          <t>Nhiều nước</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Trung binh gan han + trung binh lich su + xu the + tham chieu 2025</t>
+          <t>Trung bình gần hạn + trung bình lịch sử + xu thế + tham chiếu 2025</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Chua co tan suat 2027, dung mo hinh bo sung</t>
+          <t>Chưa có tần suất 2027, dùng mô hình bổ sung</t>
         </is>
       </c>
     </row>
@@ -941,17 +941,17 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Nhieu nuoc</t>
+          <t>Nhiều nước</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Trung binh gan han + trung binh lich su + xu the + tham chieu 2025</t>
+          <t>Trung bình gần hạn + trung bình lịch sử + xu thế + tham chiếu 2025</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Chua co tan suat 2027, dung mo hinh bo sung</t>
+          <t>Chưa có tần suất 2027, dùng mô hình bổ sung</t>
         </is>
       </c>
     </row>
@@ -986,17 +986,17 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Trung binh gan han + trung binh lich su + xu the + tham chieu 2025</t>
+          <t>Trung bình gần hạn + trung bình lịch sử + xu thế + tham chiếu 2025</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Chua co tan suat 2027, dung mo hinh bo sung</t>
+          <t>Chưa có tần suất 2027, dùng mô hình bổ sung</t>
         </is>
       </c>
     </row>
@@ -1031,17 +1031,17 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Trung binh gan han + trung binh lich su + xu the + tham chieu 2025</t>
+          <t>Trung bình gần hạn + trung bình lịch sử + xu thế + tham chiếu 2025</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Chua co tan suat 2027, dung mo hinh bo sung</t>
+          <t>Chưa có tần suất 2027, dùng mô hình bổ sung</t>
         </is>
       </c>
     </row>
@@ -11825,12 +11825,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Trung binh gan han + trung binh lich su + xu the + tham chieu 2025</t>
+          <t>Trung bình gần hạn + trung bình lịch sử + xu thế + tham chiếu 2025</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -11864,7 +11864,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Chua co tan suat 2027, dung mo hinh bo sung</t>
+          <t>Chưa có tần suất 2027, dùng mô hình bổ sung</t>
         </is>
       </c>
     </row>
@@ -11881,12 +11881,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Trung binh gan han + trung binh lich su + xu the + tham chieu 2025</t>
+          <t>Trung bình gần hạn + trung bình lịch sử + xu thế + tham chiếu 2025</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -11920,7 +11920,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Chua co tan suat 2027, dung mo hinh bo sung</t>
+          <t>Chưa có tần suất 2027, dùng mô hình bổ sung</t>
         </is>
       </c>
     </row>
@@ -11937,12 +11937,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Trung binh gan han + trung binh lich su + xu the + tham chieu 2025</t>
+          <t>Trung bình gần hạn + trung bình lịch sử + xu thế + tham chiếu 2025</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -11976,7 +11976,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Chua co tan suat 2027, dung mo hinh bo sung</t>
+          <t>Chưa có tần suất 2027, dùng mô hình bổ sung</t>
         </is>
       </c>
     </row>
@@ -11993,12 +11993,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Nhieu nuoc</t>
+          <t>Nhiều nước</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Trung binh gan han + trung binh lich su + xu the + tham chieu 2025</t>
+          <t>Trung bình gần hạn + trung bình lịch sử + xu thế + tham chiếu 2025</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -12032,7 +12032,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Chua co tan suat 2027, dung mo hinh bo sung</t>
+          <t>Chưa có tần suất 2027, dùng mô hình bổ sung</t>
         </is>
       </c>
     </row>
@@ -12049,12 +12049,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Nhieu nuoc</t>
+          <t>Nhiều nước</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Trung binh gan han + trung binh lich su + xu the + tham chieu 2025</t>
+          <t>Trung bình gần hạn + trung bình lịch sử + xu thế + tham chiếu 2025</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -12088,7 +12088,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Chua co tan suat 2027, dung mo hinh bo sung</t>
+          <t>Chưa có tần suất 2027, dùng mô hình bổ sung</t>
         </is>
       </c>
     </row>
@@ -12105,12 +12105,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Nhieu nuoc</t>
+          <t>Nhiều nước</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Trung binh gan han + trung binh lich su + xu the + tham chieu 2025</t>
+          <t>Trung bình gần hạn + trung bình lịch sử + xu thế + tham chiếu 2025</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -12144,7 +12144,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Chua co tan suat 2027, dung mo hinh bo sung</t>
+          <t>Chưa có tần suất 2027, dùng mô hình bổ sung</t>
         </is>
       </c>
     </row>
@@ -12161,12 +12161,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Nhieu nuoc</t>
+          <t>Nhiều nước</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Trung binh gan han + trung binh lich su + xu the + tham chieu 2025</t>
+          <t>Trung bình gần hạn + trung bình lịch sử + xu thế + tham chiếu 2025</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -12200,7 +12200,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Chua co tan suat 2027, dung mo hinh bo sung</t>
+          <t>Chưa có tần suất 2027, dùng mô hình bổ sung</t>
         </is>
       </c>
     </row>
@@ -12217,12 +12217,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Trung binh gan han + trung binh lich su + xu the + tham chieu 2025</t>
+          <t>Trung bình gần hạn + trung bình lịch sử + xu thế + tham chiếu 2025</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -12256,7 +12256,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Chua co tan suat 2027, dung mo hinh bo sung</t>
+          <t>Chưa có tần suất 2027, dùng mô hình bổ sung</t>
         </is>
       </c>
     </row>
@@ -12273,12 +12273,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Nhieu nuoc</t>
+          <t>Nhiều nước</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Trung binh gan han + trung binh lich su + xu the + tham chieu 2025</t>
+          <t>Trung bình gần hạn + trung bình lịch sử + xu thế + tham chiếu 2025</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -12312,7 +12312,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Chua co tan suat 2027, dung mo hinh bo sung</t>
+          <t>Chưa có tần suất 2027, dùng mô hình bổ sung</t>
         </is>
       </c>
     </row>
@@ -12329,12 +12329,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Nhieu nuoc</t>
+          <t>Nhiều nước</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Trung binh gan han + trung binh lich su + xu the + tham chieu 2025</t>
+          <t>Trung bình gần hạn + trung bình lịch sử + xu thế + tham chiếu 2025</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -12368,7 +12368,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Chua co tan suat 2027, dung mo hinh bo sung</t>
+          <t>Chưa có tần suất 2027, dùng mô hình bổ sung</t>
         </is>
       </c>
     </row>
@@ -12385,12 +12385,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Trung binh gan han + trung binh lich su + xu the + tham chieu 2025</t>
+          <t>Trung bình gần hạn + trung bình lịch sử + xu thế + tham chiếu 2025</t>
         </is>
       </c>
       <c r="G12" t="n">
@@ -12424,7 +12424,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Chua co tan suat 2027, dung mo hinh bo sung</t>
+          <t>Chưa có tần suất 2027, dùng mô hình bổ sung</t>
         </is>
       </c>
     </row>
@@ -12441,12 +12441,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Trung binh gan han + trung binh lich su + xu the + tham chieu 2025</t>
+          <t>Trung bình gần hạn + trung bình lịch sử + xu thế + tham chiếu 2025</t>
         </is>
       </c>
       <c r="G13" t="n">
@@ -12480,7 +12480,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>Chua co tan suat 2027, dung mo hinh bo sung</t>
+          <t>Chưa có tần suất 2027, dùng mô hình bổ sung</t>
         </is>
       </c>
     </row>

</xml_diff>